<commit_message>
Add Failur and Spare Parts report to aplication
</commit_message>
<xml_diff>
--- a/Obszar testowy/Awaryjność/kalkulacja Blanc PRO.xlsx
+++ b/Obszar testowy/Awaryjność/kalkulacja Blanc PRO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ReportsBI\Obszar testowy\Awaryjność\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FC7A11-F9EA-41AF-A12F-FD7092598FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C861D304-0CD3-4C4A-A890-EE4A4636FED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="źródła danych" sheetId="8" r:id="rId1"/>
@@ -15115,7 +15115,7 @@
     <col min="15" max="15" width="9.85546875" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="19.140625" customWidth="1"/>
     <col min="22" max="22" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.7109375" customWidth="1"/>
+    <col min="23" max="23" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -17988,6 +17988,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3fec9504-7640-4451-840c-8d09d21130e6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010053AB71B891A2544DBD445D04ABE7886B" ma:contentTypeVersion="11" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="323ef943dc9fb95ca33ee9e1c20c1484">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0" xmlns:ns3="3fec9504-7640-4451-840c-8d09d21130e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa2476893f5436c76bf320e2ff6b1281" ns2:_="" ns3:_="">
     <xsd:import namespace="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0"/>
@@ -18182,27 +18202,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3fec9504-7640-4451-840c-8d09d21130e6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DFC4402-E35E-46FF-8848-81414920BC84}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5150075-143E-4EB1-BF6D-1F0C09ED3DE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0"/>
+    <ds:schemaRef ds:uri="3fec9504-7640-4451-840c-8d09d21130e6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC7D9EEB-D65E-44A8-BCF5-7663D46C9A1A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18219,23 +18238,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5150075-143E-4EB1-BF6D-1F0C09ED3DE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d6c5dbd-25b1-4fbf-83f9-b289d7b111a0"/>
-    <ds:schemaRef ds:uri="3fec9504-7640-4451-840c-8d09d21130e6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DFC4402-E35E-46FF-8848-81414920BC84}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>